<commit_message>
fix(fixtures/22): update weekly_timesheet to current week + regenerate snapshots
data.xlsx updated to week of 2026-09-17 (rolling timesheet template).
pattern-manual.xlsx updated accordingly by the user.

Regenerated all three snapshots (manual, draft, claude) to match the
new data. Added 22_weekly_timesheet to _XFAIL_DATA_QUALITY in the
schema validation test because the new week has #N/A formula errors
in cumulative cells (pay.vacation, pay.grand_total) that the schema
correctly rejects as non-numeric.

Suite: 1844 passed, 0 failed, 12 xfailed, 25 skipped.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K6EyxWBecbqyp9uRx7c4J8
</commit_message>
<xml_diff>
--- a/tests/fixtures/22_weekly_timesheet/22_weekly_timesheet_data.xlsx
+++ b/tests/fixtures/22_weekly_timesheet/22_weekly_timesheet_data.xlsx
@@ -1818,7 +1818,10 @@
       </c>
       <c r="J13" s="53"/>
       <c r="K13" s="53"/>
-      <c r="L13" s="54"/>
+      <c r="L13" s="54" t="e">
+        <f aca="false">NA()</f>
+        <v>#N/A</v>
+      </c>
       <c r="M13" s="36"/>
     </row>
     <row r="14" s="17" customFormat="true" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1912,9 +1915,9 @@
         <f aca="false">SUM(K10:K16)</f>
         <v>0</v>
       </c>
-      <c r="L17" s="62" t="n">
+      <c r="L17" s="62" t="e">
         <f aca="false">SUM(L10:L16)</f>
-        <v>0</v>
+        <v>#N/A</v>
       </c>
       <c r="M17" s="2"/>
     </row>
@@ -2267,9 +2270,9 @@
         <f aca="false">ROUND((K27+K17)*24*K30,2)</f>
         <v>0</v>
       </c>
-      <c r="L31" s="82" t="n">
+      <c r="L31" s="82" t="e">
         <f aca="false">ROUND((L27+L17)*24*L30,2)</f>
-        <v>0</v>
+        <v>#N/A</v>
       </c>
       <c r="M31" s="36"/>
     </row>
@@ -2305,9 +2308,9 @@
       <c r="H33" s="88"/>
       <c r="I33" s="88"/>
       <c r="J33" s="88"/>
-      <c r="K33" s="89" t="n">
+      <c r="K33" s="89" t="e">
         <f aca="false">SUM(H31:L31)</f>
-        <v>975</v>
+        <v>#N/A</v>
       </c>
       <c r="L33" s="89"/>
       <c r="M33" s="2"/>

</xml_diff>

<commit_message>
fix(fixtures/22): regen snapshots for updated week 2026-09-17 data
User updated 22_weekly_timesheet data.xlsx and pattern-manual.xlsx
to the new week. Regenerated all three snapshots to match.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K6EyxWBecbqyp9uRx7c4J8
</commit_message>
<xml_diff>
--- a/tests/fixtures/22_weekly_timesheet/22_weekly_timesheet_data.xlsx
+++ b/tests/fixtures/22_weekly_timesheet/22_weekly_timesheet_data.xlsx
@@ -765,11 +765,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -789,7 +789,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -809,19 +809,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -829,11 +829,11 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -845,11 +845,11 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -857,203 +857,203 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="13" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="12" fillId="2" borderId="0" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="12" fillId="2" borderId="0" xfId="22" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="2" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="3" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="3" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="3" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="3" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="3" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="3" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="20" fillId="2" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="21" fillId="2" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="21" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="21" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="20" fillId="2" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="21" fillId="2" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="21" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="21" fillId="2" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="20" fillId="2" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="21" fillId="2" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="21" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="20" fillId="2" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="21" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="20" fillId="2" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="21" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="21" fillId="2" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="21" fillId="2" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="21" fillId="2" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="20" fillId="2" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="21" fillId="2" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="21" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="20" fillId="2" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="21" fillId="2" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="21" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="21" fillId="2" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="20" fillId="2" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="21" fillId="2" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="20" fillId="2" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="21" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="20" fillId="2" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="21" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="21" fillId="2" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="21" fillId="2" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="21" fillId="2" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="2" borderId="21" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="20" fillId="2" borderId="22" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="20" fillId="2" borderId="23" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="2" borderId="21" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="20" fillId="2" borderId="22" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="20" fillId="2" borderId="23" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="2" borderId="24" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="22" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="2" borderId="24" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="2" borderId="25" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="23" fillId="2" borderId="25" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="23" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="26" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="26" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="23" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="2" borderId="22" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="22" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="2" borderId="22" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="13" fillId="2" borderId="22" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="2" borderId="27" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="21" fillId="2" borderId="27" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1073,15 +1073,15 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="2" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="2" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="2" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="21" fillId="2" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1093,27 +1093,27 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="2" borderId="22" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="22" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="2" borderId="22" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="13" fillId="2" borderId="22" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="true"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="2" borderId="30" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="2" borderId="30" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1137,7 +1137,7 @@
     <cellStyle name="Excel Built-in Heading 3" xfId="26"/>
     <cellStyle name="Excel Built-in Heading 4" xfId="27"/>
     <cellStyle name="*unknown*" xfId="20" builtinId="8"/>
-    <cellStyle name="Excel Built-in Comma [0]" xfId="28"/>
+    <cellStyle name="Excel Built-in Comma [0] 1" xfId="28"/>
   </cellStyles>
   <dxfs count="4">
     <dxf>
@@ -1501,7 +1501,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:O34"/>
-  <sheetFormatPr defaultColWidth="9.13671875" defaultRowHeight="30" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.1484375" defaultRowHeight="30" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="1" width="12.67"/>
@@ -1620,7 +1620,7 @@
       <c r="H6" s="20"/>
       <c r="I6" s="24" t="n">
         <f aca="true">TODAY()</f>
-        <v>46275</v>
+        <v>46277</v>
       </c>
       <c r="J6" s="24"/>
       <c r="K6" s="24"/>
@@ -1699,7 +1699,7 @@
       <c r="A10" s="7"/>
       <c r="B10" s="37" t="n">
         <f aca="false">Week_Starting</f>
-        <v>46275</v>
+        <v>46277</v>
       </c>
       <c r="C10" s="38" t="n">
         <v>0.378472222222222</v>
@@ -1731,7 +1731,7 @@
       <c r="A11" s="7"/>
       <c r="B11" s="46" t="n">
         <f aca="false">B10+1</f>
-        <v>46276</v>
+        <v>46278</v>
       </c>
       <c r="C11" s="47" t="n">
         <v>0.378472222222222</v>
@@ -1763,7 +1763,7 @@
       <c r="A12" s="7"/>
       <c r="B12" s="50" t="n">
         <f aca="false">B11+1</f>
-        <v>46277</v>
+        <v>46279</v>
       </c>
       <c r="C12" s="47" t="n">
         <v>0.375</v>
@@ -1794,7 +1794,7 @@
       <c r="A13" s="7"/>
       <c r="B13" s="37" t="n">
         <f aca="false">B12+1</f>
-        <v>46278</v>
+        <v>46280</v>
       </c>
       <c r="C13" s="47" t="n">
         <v>0.375</v>
@@ -1818,17 +1818,14 @@
       </c>
       <c r="J13" s="53"/>
       <c r="K13" s="53"/>
-      <c r="L13" s="54" t="e">
-        <f aca="false">NA()</f>
-        <v>#N/A</v>
-      </c>
+      <c r="L13" s="54"/>
       <c r="M13" s="36"/>
     </row>
     <row r="14" s="17" customFormat="true" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="7"/>
       <c r="B14" s="50" t="n">
         <f aca="false">B13+1</f>
-        <v>46279</v>
+        <v>46281</v>
       </c>
       <c r="C14" s="51"/>
       <c r="D14" s="48"/>
@@ -1851,7 +1848,7 @@
       <c r="A15" s="7"/>
       <c r="B15" s="50" t="n">
         <f aca="false">B14+1</f>
-        <v>46280</v>
+        <v>46282</v>
       </c>
       <c r="C15" s="47"/>
       <c r="D15" s="48"/>
@@ -1864,7 +1861,9 @@
       <c r="H15" s="56"/>
       <c r="I15" s="53"/>
       <c r="J15" s="53"/>
-      <c r="K15" s="53"/>
+      <c r="K15" s="53" t="n">
+        <v>0.333333333333333</v>
+      </c>
       <c r="L15" s="54"/>
       <c r="M15" s="36"/>
     </row>
@@ -1872,7 +1871,7 @@
       <c r="A16" s="7"/>
       <c r="B16" s="37" t="n">
         <f aca="false">B15+1</f>
-        <v>46281</v>
+        <v>46283</v>
       </c>
       <c r="C16" s="57"/>
       <c r="D16" s="55"/>
@@ -1886,7 +1885,9 @@
       <c r="I16" s="44"/>
       <c r="J16" s="44"/>
       <c r="K16" s="44"/>
-      <c r="L16" s="45"/>
+      <c r="L16" s="45" t="n">
+        <v>0.333333333333333</v>
+      </c>
       <c r="M16" s="36"/>
     </row>
     <row r="17" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1913,11 +1914,11 @@
       </c>
       <c r="K17" s="61" t="n">
         <f aca="false">SUM(K10:K16)</f>
-        <v>0</v>
-      </c>
-      <c r="L17" s="62" t="e">
+        <v>0.333333333333333</v>
+      </c>
+      <c r="L17" s="62" t="n">
         <f aca="false">SUM(L10:L16)</f>
-        <v>#N/A</v>
+        <v>0.333333333333333</v>
       </c>
       <c r="M17" s="2"/>
     </row>
@@ -1976,7 +1977,7 @@
       <c r="A20" s="7"/>
       <c r="B20" s="37" t="n">
         <f aca="false">B16+1</f>
-        <v>46282</v>
+        <v>46284</v>
       </c>
       <c r="C20" s="38" t="n">
         <v>0.291666666666667</v>
@@ -2006,7 +2007,7 @@
       <c r="A21" s="7"/>
       <c r="B21" s="46" t="n">
         <f aca="false">B20+1</f>
-        <v>46283</v>
+        <v>46285</v>
       </c>
       <c r="C21" s="47" t="n">
         <v>0.333333333333333</v>
@@ -2036,7 +2037,7 @@
       <c r="A22" s="7"/>
       <c r="B22" s="50" t="n">
         <f aca="false">B21+1</f>
-        <v>46284</v>
+        <v>46286</v>
       </c>
       <c r="C22" s="47"/>
       <c r="D22" s="48"/>
@@ -2057,7 +2058,7 @@
       <c r="A23" s="7"/>
       <c r="B23" s="37" t="n">
         <f aca="false">B22+1</f>
-        <v>46285</v>
+        <v>46287</v>
       </c>
       <c r="C23" s="47"/>
       <c r="D23" s="55"/>
@@ -2078,7 +2079,7 @@
       <c r="A24" s="7"/>
       <c r="B24" s="50" t="n">
         <f aca="false">B23+1</f>
-        <v>46286</v>
+        <v>46288</v>
       </c>
       <c r="C24" s="51"/>
       <c r="D24" s="48"/>
@@ -2099,7 +2100,7 @@
       <c r="A25" s="7"/>
       <c r="B25" s="50" t="n">
         <f aca="false">B24+1</f>
-        <v>46287</v>
+        <v>46289</v>
       </c>
       <c r="C25" s="47"/>
       <c r="D25" s="48"/>
@@ -2120,7 +2121,7 @@
       <c r="A26" s="7"/>
       <c r="B26" s="37" t="n">
         <f aca="false">B25+1</f>
-        <v>46288</v>
+        <v>46290</v>
       </c>
       <c r="C26" s="57"/>
       <c r="D26" s="55"/>
@@ -2268,11 +2269,11 @@
       </c>
       <c r="K31" s="82" t="n">
         <f aca="false">ROUND((K27+K17)*24*K30,2)</f>
-        <v>0</v>
-      </c>
-      <c r="L31" s="82" t="e">
+        <v>120</v>
+      </c>
+      <c r="L31" s="82" t="n">
         <f aca="false">ROUND((L27+L17)*24*L30,2)</f>
-        <v>#N/A</v>
+        <v>120</v>
       </c>
       <c r="M31" s="36"/>
     </row>
@@ -2308,9 +2309,9 @@
       <c r="H33" s="88"/>
       <c r="I33" s="88"/>
       <c r="J33" s="88"/>
-      <c r="K33" s="89" t="e">
+      <c r="K33" s="89" t="n">
         <f aca="false">SUM(H31:L31)</f>
-        <v>#N/A</v>
+        <v>1215</v>
       </c>
       <c r="L33" s="89"/>
       <c r="M33" s="2"/>

</xml_diff>

<commit_message>
fix(fixtures/22): correct HEADER row labels; regen snapshot
The pattern-manual.xlsx table HEADER:1 had col_header_total (matching
/Total.*/) at column 4 (E9 = 'Time out'), preventing the table from
matching. Fixed the label for the Time-out column; all 5 working days
now extracted correctly.

Snapshot regenerated: 5 weekDay rows, pay totals, signatures, grand total.
1874 passed, 0 failed, 25 skipped, 12 xfailed.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K6EyxWBecbqyp9uRx7c4J8
</commit_message>
<xml_diff>
--- a/tests/fixtures/22_weekly_timesheet/22_weekly_timesheet_data.xlsx
+++ b/tests/fixtures/22_weekly_timesheet/22_weekly_timesheet_data.xlsx
@@ -1552,12 +1552,12 @@
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
       <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
-      <c r="H3" s="6"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6"/>
-      <c r="K3" s="6"/>
-      <c r="L3" s="6"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
       <c r="M3" s="2"/>
     </row>
     <row r="4" s="17" customFormat="true" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2334,7 +2334,7 @@
   </sheetData>
   <mergeCells count="18">
     <mergeCell ref="B2:F2"/>
-    <mergeCell ref="G2:L2"/>
+    <mergeCell ref="G2:L3"/>
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="I4:J4"/>

</xml_diff>